<commit_message>
Code fixed to be consistent with PyTO
</commit_message>
<xml_diff>
--- a/DataVaryingTemperature/Original_LSR_20251119_all_materials.xlsx
+++ b/DataVaryingTemperature/Original_LSR_20251119_all_materials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataVaryingTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAF33F15-E9A8-43D3-A9D3-0EFC55D20D6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{327B9C6C-91B2-4F36-8B63-0C0C02F796AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1740" yWindow="1884" windowWidth="20604" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2436" yWindow="2580" windowWidth="20604" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -607,7 +607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V18"/>
+  <dimension ref="A1:W18"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.6640625" style="1" customWidth="1"/>
@@ -620,11 +620,11 @@
     <col min="15" max="15" width="10" style="1" customWidth="1"/>
     <col min="16" max="16" width="13.6640625" style="1" customWidth="1"/>
     <col min="17" max="17" width="16.5546875" style="1" customWidth="1"/>
-    <col min="18" max="704" width="20.5546875" style="1" customWidth="1"/>
-    <col min="705" max="16384" width="9.109375" style="1"/>
+    <col min="18" max="705" width="20.5546875" style="1" customWidth="1"/>
+    <col min="706" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="3"/>
       <c r="B1" s="6" t="s">
         <v>4</v>
@@ -678,7 +678,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
       <c r="B2" s="7" t="s">
         <v>7</v>
@@ -732,7 +732,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>34</v>
       </c>
@@ -745,30 +745,28 @@
       <c r="D3" s="17">
         <v>31660210473.422401</v>
       </c>
-      <c r="E3" s="12">
-        <f>D3*EXP(-2000/Q3)</f>
-        <v>318975670.52076489</v>
-      </c>
-      <c r="F3" s="12">
-        <f>0.1*D3*EXP(-3000/Q3)</f>
-        <v>3201691.1808246872</v>
-      </c>
-      <c r="G3" s="12">
-        <v>1.0001904096107801</v>
-      </c>
-      <c r="H3" s="12">
+      <c r="E3" s="17">
+        <v>73276522231.125107</v>
+      </c>
+      <c r="F3" s="17">
+        <v>42098834999.111099</v>
+      </c>
+      <c r="G3" s="17">
+        <f>0.001*F4</f>
+        <v>2048198742.5744901</v>
+      </c>
+      <c r="H3" s="17">
         <v>168216570.304768</v>
       </c>
-      <c r="I3" s="12">
-        <f>0.1*H3*EXP(-2000/Q3)</f>
-        <v>169477.68982998349</v>
-      </c>
-      <c r="J3" s="12">
-        <f>0.1*H3*EXP(-3000/Q3)</f>
-        <v>17011.179065454031</v>
+      <c r="I3" s="17">
+        <v>1626009334.9888</v>
+      </c>
+      <c r="J3" s="17">
+        <v>1362827.91216376</v>
       </c>
       <c r="K3" s="17">
-        <v>1.0002813979562399</v>
+        <f>0.001*J3</f>
+        <v>1362.8279121637602</v>
       </c>
       <c r="L3" s="8">
         <v>161</v>
@@ -792,7 +790,7 @@
         <v>112000000</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -806,29 +804,27 @@
         <v>88122361302.941193</v>
       </c>
       <c r="E4" s="12">
-        <f t="shared" ref="E4:E5" si="0">D4*EXP(-2000/Q4)</f>
-        <v>425450353.708947</v>
+        <v>43160916887.095703</v>
       </c>
       <c r="F4" s="12">
-        <f t="shared" ref="F4:F5" si="1">0.1*D4*EXP(-3000/Q4)</f>
-        <v>2956175.8899659268</v>
-      </c>
-      <c r="G4" s="12">
-        <v>0.99968676964325098</v>
+        <v>2048198742574.49</v>
+      </c>
+      <c r="G4" s="17">
+        <f t="shared" ref="G4:G12" si="0">0.001*F5</f>
+        <v>2472842900.6711802</v>
       </c>
       <c r="H4" s="12">
         <v>331895501.95574099</v>
       </c>
       <c r="I4" s="12">
-        <f t="shared" ref="I4:I5" si="2">0.1*H4*EXP(-2000/Q4)</f>
-        <v>160237.4886619903</v>
+        <v>411398268.51887101</v>
       </c>
       <c r="J4" s="12">
-        <f t="shared" ref="J4:J5" si="3">0.1*H4*EXP(-3000/Q4)</f>
-        <v>11133.853727509615</v>
-      </c>
-      <c r="K4" s="12">
-        <v>1.00011111067342</v>
+        <v>211126489.35119501</v>
+      </c>
+      <c r="K4" s="17">
+        <f t="shared" ref="K4:K12" si="1">0.001*J4</f>
+        <v>211126.48935119502</v>
       </c>
       <c r="L4" s="8">
         <v>121</v>
@@ -852,7 +848,7 @@
         <v>118000000</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>36</v>
       </c>
@@ -866,29 +862,27 @@
         <v>92976880986.810806</v>
       </c>
       <c r="E5" s="12">
+        <v>36504792717.403801</v>
+      </c>
+      <c r="F5" s="12">
+        <v>2472842900671.1802</v>
+      </c>
+      <c r="G5" s="17">
         <f t="shared" si="0"/>
-        <v>306684777.10425931</v>
-      </c>
-      <c r="F5" s="12">
-        <f t="shared" si="1"/>
-        <v>1761371.0038603023</v>
-      </c>
-      <c r="G5" s="12">
-        <v>0.99992423656867901</v>
+        <v>171529075.34430802</v>
       </c>
       <c r="H5" s="12">
         <v>413532439.30818099</v>
       </c>
       <c r="I5" s="12">
-        <f t="shared" si="2"/>
-        <v>136403.9131325568</v>
+        <v>478670621.39346302</v>
       </c>
       <c r="J5" s="12">
-        <f t="shared" si="3"/>
-        <v>7834.0340095552874</v>
-      </c>
-      <c r="K5" s="12">
-        <v>1.0004243155682</v>
+        <v>10759114.630594</v>
+      </c>
+      <c r="K5" s="17">
+        <f t="shared" si="1"/>
+        <v>10759.114630594</v>
       </c>
       <c r="L5" s="8">
         <v>155</v>
@@ -912,7 +906,7 @@
         <v>150000000</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>37</v>
       </c>
@@ -931,8 +925,9 @@
       <c r="F6" s="12">
         <v>171529075344.30801</v>
       </c>
-      <c r="G6" s="12">
-        <v>1.0006921851331401</v>
+      <c r="G6" s="17">
+        <f t="shared" si="0"/>
+        <v>11119522273.9464</v>
       </c>
       <c r="H6" s="12">
         <v>384064916.71307498</v>
@@ -943,8 +938,9 @@
       <c r="J6" s="12">
         <v>9802478271.9358501</v>
       </c>
-      <c r="K6" s="12">
-        <v>0.99970767300819297</v>
+      <c r="K6" s="17">
+        <f t="shared" si="1"/>
+        <v>9802478.2719358504</v>
       </c>
       <c r="L6" s="8">
         <v>15</v>
@@ -967,10 +963,10 @@
       <c r="R6" s="8">
         <v>229000000</v>
       </c>
-      <c r="T6" s="5"/>
-      <c r="V6" s="5"/>
-    </row>
-    <row r="7" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+      <c r="U6" s="5"/>
+      <c r="W6" s="5"/>
+    </row>
+    <row r="7" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>38</v>
       </c>
@@ -989,8 +985,9 @@
       <c r="F7" s="12">
         <v>11119522273946.4</v>
       </c>
-      <c r="G7" s="12">
-        <v>1.0003021190852499</v>
+      <c r="G7" s="17">
+        <f t="shared" si="0"/>
+        <v>19958155949.305103</v>
       </c>
       <c r="H7" s="12">
         <v>1076144940.77356</v>
@@ -1001,8 +998,9 @@
       <c r="J7" s="12">
         <v>694123231212.5</v>
       </c>
-      <c r="K7" s="12">
-        <v>0.99944668568157702</v>
+      <c r="K7" s="17">
+        <f t="shared" si="1"/>
+        <v>694123231.21249998</v>
       </c>
       <c r="L7" s="8">
         <v>15</v>
@@ -1026,7 +1024,7 @@
         <v>229000000</v>
       </c>
     </row>
-    <row r="8" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>39</v>
       </c>
@@ -1045,8 +1043,9 @@
       <c r="F8" s="12">
         <v>19958155949305.102</v>
       </c>
-      <c r="G8" s="12">
-        <v>1.0003120524356199</v>
+      <c r="G8" s="17">
+        <f t="shared" si="0"/>
+        <v>5005582473.5935307</v>
       </c>
       <c r="H8" s="12">
         <v>1122217185.4625299</v>
@@ -1057,8 +1056,9 @@
       <c r="J8" s="12">
         <v>285480605375.97302</v>
       </c>
-      <c r="K8" s="12">
-        <v>0.99998084198200499</v>
+      <c r="K8" s="17">
+        <f t="shared" si="1"/>
+        <v>285480605.37597305</v>
       </c>
       <c r="L8" s="8">
         <v>18</v>
@@ -1082,7 +1082,7 @@
         <v>364000000</v>
       </c>
     </row>
-    <row r="9" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>40</v>
       </c>
@@ -1101,8 +1101,9 @@
       <c r="F9" s="12">
         <v>5005582473593.5303</v>
       </c>
-      <c r="G9" s="12">
-        <v>1.00279637203968</v>
+      <c r="G9" s="17">
+        <f t="shared" si="0"/>
+        <v>3667722145.0622702</v>
       </c>
       <c r="H9" s="12">
         <v>367949011.25479698</v>
@@ -1113,8 +1114,9 @@
       <c r="J9" s="12">
         <v>19124155940.442501</v>
       </c>
-      <c r="K9" s="12">
-        <v>0.99981116858122199</v>
+      <c r="K9" s="17">
+        <f t="shared" si="1"/>
+        <v>19124155.940442502</v>
       </c>
       <c r="L9" s="8">
         <v>13</v>
@@ -1138,7 +1140,7 @@
         <v>407000000</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>41</v>
       </c>
@@ -1157,8 +1159,9 @@
       <c r="F10" s="12">
         <v>3667722145062.27</v>
       </c>
-      <c r="G10" s="12">
-        <v>1.00055405463834</v>
+      <c r="G10" s="17">
+        <f t="shared" si="0"/>
+        <v>175213569.92829001</v>
       </c>
       <c r="H10" s="12">
         <v>1223876264.4957099</v>
@@ -1169,8 +1172,9 @@
       <c r="J10" s="12">
         <v>26710952266.052299</v>
       </c>
-      <c r="K10" s="12">
-        <v>1.0003928619167901</v>
+      <c r="K10" s="17">
+        <f t="shared" si="1"/>
+        <v>26710952.266052298</v>
       </c>
       <c r="L10" s="8">
         <v>10</v>
@@ -1194,7 +1198,7 @@
         <v>485000000</v>
       </c>
     </row>
-    <row r="11" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>42</v>
       </c>
@@ -1213,8 +1217,9 @@
       <c r="F11" s="12">
         <v>175213569928.29001</v>
       </c>
-      <c r="G11" s="12">
-        <v>1.0007894571356</v>
+      <c r="G11" s="17">
+        <f t="shared" si="0"/>
+        <v>13930248415.001699</v>
       </c>
       <c r="H11" s="12">
         <v>425435242.49228698</v>
@@ -1225,8 +1230,9 @@
       <c r="J11" s="12">
         <v>751102621.40532196</v>
       </c>
-      <c r="K11" s="12">
-        <v>0.99976714584067305</v>
+      <c r="K11" s="17">
+        <f t="shared" si="1"/>
+        <v>751102.62140532199</v>
       </c>
       <c r="L11" s="8">
         <v>17</v>
@@ -1250,7 +1256,7 @@
         <v>245000000</v>
       </c>
     </row>
-    <row r="12" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>43</v>
       </c>
@@ -1269,8 +1275,9 @@
       <c r="F12" s="12">
         <v>13930248415001.699</v>
       </c>
-      <c r="G12" s="12">
-        <v>1.0010307445001101</v>
+      <c r="G12" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="H12" s="12">
         <v>504059502.99034601</v>
@@ -1281,8 +1288,9 @@
       <c r="J12" s="12">
         <v>8072139562.2192097</v>
       </c>
-      <c r="K12" s="12">
-        <v>1.0002667881887199</v>
+      <c r="K12" s="17">
+        <f t="shared" si="1"/>
+        <v>8072139.56221921</v>
       </c>
       <c r="L12" s="8">
         <v>17</v>
@@ -1306,7 +1314,7 @@
         <v>245000000</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B16" s="13"/>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.3">

</xml_diff>